<commit_message>
Sync working branch with main: DRHP offer share-structure extraction
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iqmpMYA81W4K2ET9so5AG
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AG6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -438,23 +438,29 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="15" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="29" max="29"/>
+    <col width="15" customWidth="1" min="30" max="30"/>
+    <col width="11" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,85 +516,115 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Fresh Shares</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>OFS Shares</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Total Shares</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Face Value</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Market Cap (Cr)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Issue/MktCap %</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Revenue FY25 (Cr)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Rev Growth %</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>PAT FY25 (Cr)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>PAT Growth %</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>PAT Margin %</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>EBITDA Margin %</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>ROE %</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>ROCE %</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Debt/Equity</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Promoter %</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Stamps</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Data Source</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>SEBI URL</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>DRHP PDF</t>
         </is>
@@ -631,51 +667,63 @@
         </is>
       </c>
       <c r="K2" t="n">
+        <v>16084000</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1807000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>17891000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q2" t="n">
         <v>819.24</v>
       </c>
-      <c r="L2" t="n">
+      <c r="R2" t="n">
         <v>30.1</v>
       </c>
-      <c r="M2" t="n">
+      <c r="S2" t="n">
         <v>52.95</v>
       </c>
-      <c r="N2" t="n">
+      <c r="T2" t="n">
         <v>12.78</v>
       </c>
-      <c r="O2" t="n">
+      <c r="U2" t="n">
         <v>6.45</v>
       </c>
-      <c r="P2" t="n">
+      <c r="V2" t="n">
         <v>13.24</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="W2" t="n">
         <v>27.59</v>
       </c>
-      <c r="U2" t="n">
+      <c r="AA2" t="n">
         <v>48.7</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>DIG DEEPER</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>FILED_THIS_WEEK</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>DRHP_PDF, derived</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr">
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/sky-alloys-and-power-limited-drhp_102415.html</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/Sky%20Alloys%20and%20Power%20Limited%20-%20Abri_p.pdf</t>
         </is>
@@ -717,49 +765,52 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
         <v>6252.83</v>
       </c>
-      <c r="L3" t="n">
+      <c r="R3" t="n">
         <v>16.03</v>
       </c>
-      <c r="M3" t="n">
+      <c r="S3" t="n">
         <v>244.82</v>
       </c>
-      <c r="N3" t="n">
+      <c r="T3" t="n">
         <v>6.64</v>
       </c>
-      <c r="O3" t="n">
+      <c r="U3" t="n">
         <v>3.87</v>
       </c>
-      <c r="P3" t="n">
+      <c r="V3" t="n">
         <v>15.25</v>
       </c>
-      <c r="U3" t="n">
+      <c r="AA3" t="n">
         <v>32</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>DIG DEEPER</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>DRHP_PDF, derived</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr">
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/oravel-stays-limited-udrhp-i_102455.html</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/ORAVEL%20STAYS%20LIMITED%20-%20Abridged_p.pdf</t>
         </is>
@@ -801,61 +852,67 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
+        <v>7282300</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="n">
         <v>1628.83</v>
       </c>
-      <c r="L4" t="n">
+      <c r="R4" t="n">
         <v>9.25</v>
       </c>
-      <c r="M4" t="n">
+      <c r="S4" t="n">
         <v>14.29</v>
       </c>
-      <c r="N4" t="n">
+      <c r="T4" t="n">
         <v>-10.71</v>
       </c>
-      <c r="O4" t="n">
+      <c r="U4" t="n">
         <v>0.87</v>
       </c>
-      <c r="P4" t="n">
+      <c r="V4" t="n">
         <v>2.18</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="W4" t="n">
         <v>12.15</v>
       </c>
-      <c r="R4" t="n">
+      <c r="X4" t="n">
         <v>12.54</v>
       </c>
-      <c r="S4" t="n">
+      <c r="Y4" t="n">
         <v>1.57</v>
       </c>
-      <c r="T4" t="n">
+      <c r="Z4" t="n">
         <v>98.48999999999999</v>
       </c>
-      <c r="U4" t="n">
+      <c r="AA4" t="n">
         <v>26.7</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>DIG DEEPER</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>FILED_THIS_WEEK</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>DRHP_PDF, derived</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr">
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/ujin-pharma-ltd-drhp_102424.html</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/Ujin%20Pharma%20Ltd.%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
@@ -892,23 +949,23 @@
           <t>Jewellery</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>INSUFFICIENT</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>FILED_THIS_WEEK</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr">
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/advit-jewels-limited-prospectus_102425.html</t>
         </is>
@@ -945,23 +1002,23 @@
           <t>Fintech</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>INSUFFICIENT</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>FILED_THIS_WEEK</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr">
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/turtlemint-fintech-solutions-limited-prospectus_102393.html</t>
         </is>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-07-13)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -633,12 +633,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sky Alloys and Power Limited</t>
+          <t>TMC Transformers India Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -653,54 +653,45 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>16084000</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1807000</v>
-      </c>
-      <c r="M2" t="n">
-        <v>17891000</v>
+          <t>Fresh</t>
+        </is>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>819.24</v>
+        <v>417.24</v>
       </c>
       <c r="R2" t="n">
-        <v>30.1</v>
+        <v>53.57</v>
       </c>
       <c r="S2" t="n">
-        <v>52.95</v>
+        <v>95.70999999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>12.78</v>
+        <v>105.19</v>
       </c>
       <c r="U2" t="n">
-        <v>6.45</v>
+        <v>22.94</v>
       </c>
       <c r="V2" t="n">
-        <v>13.24</v>
+        <v>31.89</v>
       </c>
       <c r="W2" t="n">
-        <v>27.59</v>
+        <v>62.28</v>
       </c>
       <c r="AA2" t="n">
-        <v>48.7</v>
+        <v>71.2</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -720,29 +711,29 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/sky-alloys-and-power-limited-drhp_102415.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/tmc-transformers-india-limited-drhp_102680.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/Sky%20Alloys%20and%20Power%20Limited%20-%20Abri_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/TMC%20Transformers%20India%20Limited%20-%20Abri_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Oravel Stays Limited</t>
+          <t>Ratnadeep Retail Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -757,7 +748,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Hospitality</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -769,25 +760,28 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>6252.83</v>
+        <v>2223.14</v>
       </c>
       <c r="R3" t="n">
-        <v>16.03</v>
+        <v>11.84</v>
       </c>
       <c r="S3" t="n">
-        <v>244.82</v>
-      </c>
-      <c r="T3" t="n">
-        <v>6.64</v>
+        <v>36.7</v>
       </c>
       <c r="U3" t="n">
-        <v>3.87</v>
+        <v>1.65</v>
       </c>
       <c r="V3" t="n">
-        <v>15.25</v>
+        <v>5.01</v>
+      </c>
+      <c r="W3" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="X3" t="n">
+        <v>17.82</v>
       </c>
       <c r="AA3" t="n">
-        <v>32</v>
+        <v>41.9</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -796,7 +790,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -807,24 +801,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/oravel-stays-limited-udrhp-i_102455.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/ratnadeep-retail-limited-drhp_102720.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/ORAVEL%20STAYS%20LIMITED%20-%20Abridged_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Ratnadeep%20Retail%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ujin Pharma Ltd.</t>
+          <t>Innoterra Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -839,12 +833,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -853,47 +847,29 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>7282300</v>
+        <v>7055315</v>
       </c>
       <c r="N4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q4" t="n">
-        <v>1628.83</v>
+        <v>163.47</v>
       </c>
       <c r="R4" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="S4" t="n">
-        <v>14.29</v>
-      </c>
-      <c r="T4" t="n">
-        <v>-10.71</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.87</v>
+        <v>-14.74</v>
       </c>
       <c r="V4" t="n">
-        <v>2.18</v>
+        <v>-6.38</v>
       </c>
       <c r="W4" t="n">
-        <v>12.15</v>
-      </c>
-      <c r="X4" t="n">
-        <v>12.54</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>98.48999999999999</v>
+        <v>1.01</v>
       </c>
       <c r="AA4" t="n">
-        <v>26.7</v>
+        <v>1.1</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -909,44 +885,39 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/ujin-pharma-ltd-drhp_102424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/innoterra-limited-drhp_102678.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/Ujin%20Pharma%20Ltd.%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/INNOTERRA%20LIMITED%20-%20Abri_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Advit Jewels Limited</t>
+          <t>Cult.Fit Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -967,19 +938,19 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/advit-jewels-limited-prospectus_102425.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/cult-fit-limited-drhp_102714.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Turtlemint Fintech Solutions Limited</t>
+          <t>Waterways Leisure Tourism Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -994,12 +965,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Fintech</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1020,7 +986,7 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/turtlemint-fintech-solutions-limited-prospectus_102393.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/waterways-leisure-tourism-limited-prospectus_102629.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy: bring the redesigned dashboard + current data to the deploy branch
The site deploys from this (default) branch, so sync index.html, assets and
data from main — where the Weekly Monitor / Pipeline / Archive redesign and the
2026-07-13 data live — so the live dashboard actually reflects main.
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -633,12 +633,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sky Alloys and Power Limited</t>
+          <t>TMC Transformers India Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -653,54 +653,45 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>16084000</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1807000</v>
-      </c>
-      <c r="M2" t="n">
-        <v>17891000</v>
+          <t>Fresh</t>
+        </is>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>819.24</v>
+        <v>417.24</v>
       </c>
       <c r="R2" t="n">
-        <v>30.1</v>
+        <v>53.57</v>
       </c>
       <c r="S2" t="n">
-        <v>52.95</v>
+        <v>95.70999999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>12.78</v>
+        <v>105.19</v>
       </c>
       <c r="U2" t="n">
-        <v>6.45</v>
+        <v>22.94</v>
       </c>
       <c r="V2" t="n">
-        <v>13.24</v>
+        <v>31.89</v>
       </c>
       <c r="W2" t="n">
-        <v>27.59</v>
+        <v>62.28</v>
       </c>
       <c r="AA2" t="n">
-        <v>48.7</v>
+        <v>71.2</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -720,29 +711,29 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/sky-alloys-and-power-limited-drhp_102415.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/tmc-transformers-india-limited-drhp_102680.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/Sky%20Alloys%20and%20Power%20Limited%20-%20Abri_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/TMC%20Transformers%20India%20Limited%20-%20Abri_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Oravel Stays Limited</t>
+          <t>Ratnadeep Retail Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -757,7 +748,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Hospitality</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -769,25 +760,28 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>6252.83</v>
+        <v>2223.14</v>
       </c>
       <c r="R3" t="n">
-        <v>16.03</v>
+        <v>11.84</v>
       </c>
       <c r="S3" t="n">
-        <v>244.82</v>
-      </c>
-      <c r="T3" t="n">
-        <v>6.64</v>
+        <v>36.7</v>
       </c>
       <c r="U3" t="n">
-        <v>3.87</v>
+        <v>1.65</v>
       </c>
       <c r="V3" t="n">
-        <v>15.25</v>
+        <v>5.01</v>
+      </c>
+      <c r="W3" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="X3" t="n">
+        <v>17.82</v>
       </c>
       <c r="AA3" t="n">
-        <v>32</v>
+        <v>41.9</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -796,7 +790,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -807,24 +801,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/oravel-stays-limited-udrhp-i_102455.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/ratnadeep-retail-limited-drhp_102720.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/ORAVEL%20STAYS%20LIMITED%20-%20Abridged_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Ratnadeep%20Retail%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ujin Pharma Ltd.</t>
+          <t>Innoterra Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -839,12 +833,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -853,47 +847,29 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>7282300</v>
+        <v>7055315</v>
       </c>
       <c r="N4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q4" t="n">
-        <v>1628.83</v>
+        <v>163.47</v>
       </c>
       <c r="R4" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="S4" t="n">
-        <v>14.29</v>
-      </c>
-      <c r="T4" t="n">
-        <v>-10.71</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.87</v>
+        <v>-14.74</v>
       </c>
       <c r="V4" t="n">
-        <v>2.18</v>
+        <v>-6.38</v>
       </c>
       <c r="W4" t="n">
-        <v>12.15</v>
-      </c>
-      <c r="X4" t="n">
-        <v>12.54</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>98.48999999999999</v>
+        <v>1.01</v>
       </c>
       <c r="AA4" t="n">
-        <v>26.7</v>
+        <v>1.1</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -909,44 +885,39 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/ujin-pharma-ltd-drhp_102424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/innoterra-limited-drhp_102678.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jun-2026/Ujin%20Pharma%20Ltd.%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/INNOTERRA%20LIMITED%20-%20Abri_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Advit Jewels Limited</t>
+          <t>Cult.Fit Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -967,19 +938,19 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/advit-jewels-limited-prospectus_102425.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/cult-fit-limited-drhp_102714.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Turtlemint Fintech Solutions Limited</t>
+          <t>Waterways Leisure Tourism Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -994,12 +965,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Fintech</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1020,7 +986,7 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jun-2026/turtlemint-fintech-solutions-limited-prospectus_102393.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/waterways-leisure-tourism-limited-prospectus_102629.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-07-20)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TMC Transformers India Limited</t>
+          <t>Gni Infrastructure Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -724,40 +724,52 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Fresh</t>
-        </is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>21029642</v>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>417.24</v>
+        <v>309.07</v>
       </c>
       <c r="R2" t="n">
-        <v>53.57</v>
+        <v>69.73</v>
       </c>
       <c r="S2" t="n">
-        <v>95.70999999999999</v>
+        <v>76.12</v>
       </c>
       <c r="T2" t="n">
-        <v>105.19</v>
+        <v>62.09</v>
       </c>
       <c r="U2" t="n">
-        <v>22.94</v>
+        <v>22.5</v>
       </c>
       <c r="V2" t="n">
-        <v>31.89</v>
+        <v>35.15</v>
       </c>
       <c r="W2" t="n">
-        <v>62.28</v>
+        <v>25.25</v>
+      </c>
+      <c r="X2" t="n">
+        <v>20.34</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>89.12</v>
       </c>
       <c r="AA2" t="n">
-        <v>71.2</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -777,44 +789,44 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/tmc-transformers-india-limited-drhp_102680.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/gni-infrastructure-limited-drhp_102874.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/TMC%20Transformers%20India%20Limited%20-%20Abri_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/GNI%20INFRASTRUCTURE%20LIMITED%20-%20DA_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ratnadeep Retail Limited</t>
+          <t>Laser Power and Infra Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -823,31 +835,31 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q3" t="n">
-        <v>2223.14</v>
+        <v>202.6</v>
       </c>
       <c r="R3" t="n">
-        <v>11.84</v>
+        <v>0.05</v>
       </c>
       <c r="S3" t="n">
-        <v>36.7</v>
+        <v>151.59</v>
+      </c>
+      <c r="T3" t="n">
+        <v>42</v>
       </c>
       <c r="U3" t="n">
-        <v>1.65</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="V3" t="n">
-        <v>5.01</v>
+        <v>148.79</v>
       </c>
       <c r="W3" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="X3" t="n">
-        <v>17.82</v>
+        <v>23.32</v>
       </c>
       <c r="AA3" t="n">
-        <v>41.9</v>
+        <v>49.6</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -867,75 +879,81 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/ratnadeep-retail-limited-drhp_102720.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/laser-power-and-infra-limited-prospectus_102821.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Ratnadeep%20Retail%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Laser%20Power%20and%20Infra%20Limited%20-%20ABr_p.pdf</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Laser Power &amp; Infra Ltd.</t>
+        </is>
+      </c>
+      <c r="AI3" t="n">
+        <v>4058</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>17.36</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>38.74</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>43.27</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>16.82</v>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/laser-power-infra-ltd</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Innoterra Limited</t>
+          <t>SBI Funds Management Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>IT Services</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>7055315</v>
-      </c>
-      <c r="N4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>163.47</v>
-      </c>
-      <c r="R4" t="n">
-        <v>-14.74</v>
-      </c>
-      <c r="V4" t="n">
-        <v>-6.38</v>
-      </c>
-      <c r="W4" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>1.1</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -945,45 +963,67 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/innoterra-limited-drhp_102678.html</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/INNOTERRA%20LIMITED%20-%20Abri_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/sbi-funds-management-limited-prospectus_102917.html</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>SBI Funds Management Ltd</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>41.62</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>140.11</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/sbi-funds-management-ipo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cult.Fit Limited</t>
+          <t>Behari Lal Engineering Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -993,7 +1033,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -1004,19 +1044,19 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/cult-fit-limited-drhp_102714.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/behari-lal-engineering-limited-corrigendum-to-drhp_102871.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Waterways Leisure Tourism Limited</t>
+          <t>Kusumgar Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1052,44 +1092,38 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/waterways-leisure-tourism-limited-prospectus_102629.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/kusumgar-limited-prospectus_102792.html</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Waterways Leisure Tourism Ltd.</t>
+          <t>Kusumgar Ltd.</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>6210</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>65.01000000000001</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>1.47</v>
+        <v>6046</v>
       </c>
       <c r="AL6" t="n">
-        <v>89.34999999999999</v>
+        <v>75.01000000000001</v>
       </c>
       <c r="AM6" t="n">
-        <v>1.44</v>
+        <v>127.89</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.6899999999999999</v>
+        <v>284.1</v>
       </c>
       <c r="AO6" t="n">
-        <v>1.17</v>
+        <v>164.57</v>
       </c>
       <c r="AP6" t="n">
-        <v>4.12</v>
+        <v>24.94</v>
       </c>
       <c r="AQ6" t="n">
-        <v>-15.72</v>
+        <v>35.8</v>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/waterways-leisure-tourism-ltd</t>
+          <t>https://groww.in/stocks/kusumgar-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-07-27)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR6"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,114 +699,60 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gni Infrastructure Limited</t>
+          <t>Fusion CX Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>21029642</v>
-      </c>
-      <c r="N2" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>309.07</v>
-      </c>
-      <c r="R2" t="n">
-        <v>69.73</v>
-      </c>
-      <c r="S2" t="n">
-        <v>76.12</v>
-      </c>
-      <c r="T2" t="n">
-        <v>62.09</v>
-      </c>
-      <c r="U2" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="V2" t="n">
-        <v>35.15</v>
-      </c>
-      <c r="W2" t="n">
-        <v>25.25</v>
-      </c>
-      <c r="X2" t="n">
-        <v>20.34</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>89.12</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>83.09999999999999</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/gni-infrastructure-limited-drhp_102874.html</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/GNI%20INFRASTRUCTURE%20LIMITED%20-%20DA_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/fusion-cx-limited-addendum-to-drhp_102992.html</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Laser Power and Infra Limited</t>
+          <t>Caliber Mining And Logistics Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -821,309 +767,70 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>202.6</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="S3" t="n">
-        <v>151.59</v>
-      </c>
-      <c r="T3" t="n">
-        <v>42</v>
-      </c>
-      <c r="U3" t="n">
-        <v>74.81999999999999</v>
-      </c>
-      <c r="V3" t="n">
-        <v>148.79</v>
-      </c>
-      <c r="W3" t="n">
-        <v>23.32</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>49.6</v>
+          <t>Mining</t>
+        </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/laser-power-and-infra-limited-prospectus_102821.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Laser%20Power%20and%20Infra%20Limited%20-%20ABr_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/caliber-mining-and-logistics-limited-prospectus_102990.html</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>Laser Power &amp; Infra Ltd.</t>
+          <t>Caliber Mining and Logistics Ltd.</t>
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>4058</v>
+        <v>3455</v>
       </c>
       <c r="AJ3" t="n">
-        <v>17.36</v>
+        <v>24.38</v>
       </c>
       <c r="AK3" t="n">
-        <v>1.2</v>
+        <v>1.73</v>
       </c>
       <c r="AL3" t="n">
-        <v>75.3</v>
+        <v>74.18000000000001</v>
       </c>
       <c r="AM3" t="n">
-        <v>38.74</v>
+        <v>146.41</v>
       </c>
       <c r="AN3" t="n">
-        <v>92.25</v>
+        <v>240.71</v>
       </c>
       <c r="AO3" t="n">
-        <v>43.27</v>
+        <v>267.23</v>
       </c>
       <c r="AP3" t="n">
-        <v>6.21</v>
+        <v>40.75</v>
       </c>
       <c r="AQ3" t="n">
-        <v>16.82</v>
+        <v>17.98</v>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/laser-power-infra-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SBI Funds Management Limited</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/sbi-funds-management-limited-prospectus_102917.html</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>SBI Funds Management Ltd</t>
-        </is>
-      </c>
-      <c r="AM4" t="n">
-        <v>41.62</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>140.11</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/sbi-funds-management-ipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Behari Lal Engineering Limited</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Corrigendum</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/behari-lal-engineering-limited-corrigendum-to-drhp_102871.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Kusumgar Limited</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/kusumgar-limited-prospectus_102792.html</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>Kusumgar Ltd.</t>
-        </is>
-      </c>
-      <c r="AI6" t="n">
-        <v>6046</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>75.01000000000001</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>127.89</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>284.1</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>164.57</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/kusumgar-ltd</t>
+          <t>https://groww.in/stocks/caliber-mining-and-logistics-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-08-03)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AR11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,17 +699,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fusion CX Limited</t>
+          <t>Indian Gas Exchange Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -719,118 +719,766 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>16710000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>61</v>
+      </c>
+      <c r="R2" t="n">
+        <v>25.01</v>
+      </c>
+      <c r="S2" t="n">
+        <v>42.02</v>
+      </c>
+      <c r="T2" t="n">
+        <v>36.47</v>
+      </c>
+      <c r="U2" t="n">
+        <v>49.53</v>
+      </c>
+      <c r="V2" t="n">
+        <v>96.06999999999999</v>
+      </c>
+      <c r="W2" t="n">
+        <v>25.72</v>
+      </c>
+      <c r="X2" t="n">
+        <v>31.71</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>80.5</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/fusion-cx-limited-addendum-to-drhp_102992.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/indian-gas-exchange-limited-drhp_102988.html</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Indian%20Gas%20Exchange%20Limited_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Caliber Mining And Logistics Limited</t>
+          <t>Yogiji Digi Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Mining</t>
-        </is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>514.0599999999999</v>
+      </c>
+      <c r="N3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>626.11</v>
+      </c>
+      <c r="R3" t="n">
+        <v>30.53</v>
+      </c>
+      <c r="S3" t="n">
+        <v>40.42</v>
+      </c>
+      <c r="T3" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="U3" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="V3" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="W3" t="n">
+        <v>21.31</v>
+      </c>
+      <c r="X3" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>66.8</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/caliber-mining-and-logistics-limited-prospectus_102990.html</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>Caliber Mining and Logistics Ltd.</t>
-        </is>
-      </c>
-      <c r="AI3" t="n">
-        <v>3455</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>24.38</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>74.18000000000001</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>146.41</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>240.71</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>267.23</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>40.75</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>17.98</v>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/caliber-mining-and-logistics-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/yogiji-digi-limited-drhp_103106.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/YOGIJI%20DIGI%20LIMITED_p.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Hero Motors Limited</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hero-motors-limited-corrigendum-to-drhp_103180.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Manipal Health Enterprises Limited</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Healthcare Services</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/manipal-health-enterprises-limited-prospectus_103300.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Master Chains N Jewels Limited</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/master-chains-n-jewels-limited_103287.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Propshop Events and Exhibitions Limited</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/propshop-events-and-exhibitions-limited-prospectus_103111.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Propshop Events And Exhibitions Ltd.</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>55.86</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/propshop-events-and-exhibitions-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Xtranet Technologies Limited</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>IT Services</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/xtranet-technologies-limited-prospectus_103105.html</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Xtranet Technologies Ltd.</t>
+        </is>
+      </c>
+      <c r="AI8" t="n">
+        <v>662</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>62.62</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>12.13</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>26.59</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/xtranet-technologies-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Aastha Spintex Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Textiles</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Textiles</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/aastha-spintex-limited-prospectus_103092.html</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Aastha Spintex Ltd.</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>336</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>53.21</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>-4.41</v>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/aastha-spintex-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lohia Corp Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/lohia-corp-limited-prospectus_103075.html</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Lohia Corp Ltd.</t>
+        </is>
+      </c>
+      <c r="AI10" t="n">
+        <v>5651</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>37.07</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/lohia-corp-ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Indo-MIM Limited</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/indo-mim-limited_103050.html</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>INDO-MIM Ltd.</t>
+        </is>
+      </c>
+      <c r="AI11" t="n">
+        <v>38273</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>77.65000000000001</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>72.29000000000001</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>204.34</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>50.61</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>44.33</v>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/indomim-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-08-10)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR11"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,12 +699,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Indian Gas Exchange Limited</t>
+          <t>Advanced Sys-Tek Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,51 +719,51 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>Auto Components</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="L2" t="n">
-        <v>16710000</v>
       </c>
       <c r="N2" t="n">
         <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>61</v>
+        <v>302.25</v>
       </c>
       <c r="R2" t="n">
-        <v>25.01</v>
+        <v>19.57</v>
       </c>
       <c r="S2" t="n">
-        <v>42.02</v>
+        <v>36.73</v>
       </c>
       <c r="T2" t="n">
-        <v>36.47</v>
+        <v>33.11</v>
       </c>
       <c r="U2" t="n">
-        <v>49.53</v>
+        <v>11.88</v>
       </c>
       <c r="V2" t="n">
-        <v>96.06999999999999</v>
+        <v>14.36</v>
       </c>
       <c r="W2" t="n">
-        <v>25.72</v>
+        <v>15.85</v>
       </c>
       <c r="X2" t="n">
-        <v>31.71</v>
+        <v>21.69</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>40.86</v>
       </c>
       <c r="AA2" t="n">
-        <v>80.5</v>
+        <v>60.8</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -783,24 +783,24 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/indian-gas-exchange-limited-drhp_102988.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/advanced-sys-tek-limited-drhp_103353.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/Indian%20Gas%20Exchange%20Limited_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Advanced%20Sys-Tek%20Limited%20%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Yogiji Digi Limited</t>
+          <t>Encube Ethicals Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -815,55 +815,37 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>514.0599999999999</v>
+          <t>OFS</t>
+        </is>
       </c>
       <c r="N3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>626.11</v>
+        <v>202.4</v>
       </c>
       <c r="R3" t="n">
-        <v>30.53</v>
-      </c>
-      <c r="S3" t="n">
-        <v>40.42</v>
-      </c>
-      <c r="T3" t="n">
-        <v>44.17</v>
-      </c>
-      <c r="U3" t="n">
-        <v>6.46</v>
+        <v>-0.1</v>
       </c>
       <c r="V3" t="n">
-        <v>10.81</v>
-      </c>
-      <c r="W3" t="n">
-        <v>21.31</v>
-      </c>
-      <c r="X3" t="n">
-        <v>17.7</v>
+        <v>0.02</v>
       </c>
       <c r="AA3" t="n">
-        <v>66.8</v>
+        <v>0.6</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -879,606 +861,12 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/yogiji-digi-limited-drhp_103106.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/encube-ethicals-limited-drhp_103383.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/jul-2026/YOGIJI%20DIGI%20LIMITED_p.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Hero Motors Limited</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Corrigendum</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hero-motors-limited-corrigendum-to-drhp_103180.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Manipal Health Enterprises Limited</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Healthcare Services</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/manipal-health-enterprises-limited-prospectus_103300.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Master Chains N Jewels Limited</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/master-chains-n-jewels-limited_103287.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Propshop Events and Exhibitions Limited</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/propshop-events-and-exhibitions-limited-prospectus_103111.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Propshop Events And Exhibitions Ltd.</t>
-        </is>
-      </c>
-      <c r="AI7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>55.86</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>1.37</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>1.31</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>-20</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/propshop-events-and-exhibitions-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Xtranet Technologies Limited</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>IT Services</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/xtranet-technologies-limited-prospectus_103105.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Xtranet Technologies Ltd.</t>
-        </is>
-      </c>
-      <c r="AI8" t="n">
-        <v>662</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>62.62</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>12.13</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>7.13</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>26.59</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>8.789999999999999</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>7.09</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/xtranet-technologies-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Aastha Spintex Limited</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Textiles</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Textiles</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/aastha-spintex-limited-prospectus_103092.html</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>Aastha Spintex Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>336</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>53.21</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>7.61</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>-4.41</v>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/aastha-spintex-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Lohia Corp Limited</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/lohia-corp-limited-prospectus_103075.html</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Lohia Corp Ltd.</t>
-        </is>
-      </c>
-      <c r="AI10" t="n">
-        <v>5651</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>37.07</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>68.66</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>7.21</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>9.109999999999999</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>6.77</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>8.470000000000001</v>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lohia-corp-ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Indo-MIM Limited</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/jul-2026/indo-mim-limited_103050.html</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>INDO-MIM Ltd.</t>
-        </is>
-      </c>
-      <c r="AI11" t="n">
-        <v>38273</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>77.65000000000001</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>72.29000000000001</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>204.34</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>50.61</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>44.33</v>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/indomim-ltd</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Encube%20Ethicals%20Limited%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-08-17)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Advanced Sys-Tek Limited</t>
+          <t>Alpine Texworld Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Auto Components</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -732,38 +732,29 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>10</v>
-      </c>
       <c r="Q2" t="n">
-        <v>302.25</v>
+        <v>342.71</v>
       </c>
       <c r="R2" t="n">
-        <v>19.57</v>
+        <v>44.41</v>
       </c>
       <c r="S2" t="n">
-        <v>36.73</v>
+        <v>21.72</v>
       </c>
       <c r="T2" t="n">
-        <v>33.11</v>
+        <v>151.75</v>
       </c>
       <c r="U2" t="n">
-        <v>11.88</v>
+        <v>6.34</v>
       </c>
       <c r="V2" t="n">
-        <v>14.36</v>
+        <v>13.84</v>
       </c>
       <c r="W2" t="n">
-        <v>15.85</v>
-      </c>
-      <c r="X2" t="n">
-        <v>21.69</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>40.86</v>
+        <v>29.44</v>
       </c>
       <c r="AA2" t="n">
-        <v>60.8</v>
+        <v>57.4</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -783,36 +774,73 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/advanced-sys-tek-limited-drhp_103353.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/alpine-texworld-limited-prospectus_103604.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Advanced%20Sys-Tek%20Limited%20%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Abridged%20prospectus_p.pdf</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Alpine Texworld Ltd.</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>224</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>29.44</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>68.56</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/alpine-texworld-ltd</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Encube Ethicals Limited</t>
+          <t>AGS Health Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Healthcare</t>
@@ -820,37 +848,52 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Healthcare Services</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>OFS</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>202.4</v>
+        <v>2041.42</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.1</v>
+        <v>70.84999999999999</v>
+      </c>
+      <c r="S3" t="n">
+        <v>206.95</v>
+      </c>
+      <c r="T3" t="n">
+        <v>44.79</v>
+      </c>
+      <c r="U3" t="n">
+        <v>10.14</v>
       </c>
       <c r="V3" t="n">
-        <v>0.02</v>
+        <v>4</v>
+      </c>
+      <c r="W3" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.6</v>
+        <v>54.6</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -861,12 +904,406 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/encube-ethicals-limited-drhp_103383.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/ags-health-limited-udrhp_103617.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Encube%20Ethicals%20Limited%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/AGS%20Health%20Limited%20-%20AP_p.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Zetwerk Manufacturing Businesses Limited</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>96837455</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>15913.32</v>
+      </c>
+      <c r="R4" t="n">
+        <v>40.43</v>
+      </c>
+      <c r="V4" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="W4" t="n">
+        <v>21.11</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>DIG DEEPER</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>DRHP_PDF, derived</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/zetwerk-manufacturing-businesses-limited-udrhp_103643.html</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Zetwerk%20Manufacturing%20Businesses%20Limited%20-%20DAP_p.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beauty Garage Limited</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-99.79000000000001</v>
+      </c>
+      <c r="V5" t="n">
+        <v>43.33</v>
+      </c>
+      <c r="W5" t="n">
+        <v>55.04</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>MONITOR</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>DRHP_PDF, derived</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/beauty-garage-limited-drhp_103479.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/BEAUTY%20GARAGE%20LIMITED%20-%20AP_p.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tonbo Imaging India Limited</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/tonbo-imaging-india-limited_103625.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sillverton Industries Limited</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/sillverton-industries-limited-addendum-ii_103621.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>J Pan Tubular Components Limited</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/j-pan-tubular-components-limited_103499.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LEAP India Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/leap-india-limited-prospectus_103511.html</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Leap India Ltd.</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>6392</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>55.64</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/leap-india-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-08-24)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alpine Texworld Limited</t>
+          <t>Tablespace Technologies Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>IT Services</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -732,29 +732,17 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
       <c r="Q2" t="n">
-        <v>342.71</v>
+        <v>2262.29</v>
       </c>
       <c r="R2" t="n">
-        <v>44.41</v>
-      </c>
-      <c r="S2" t="n">
-        <v>21.72</v>
-      </c>
-      <c r="T2" t="n">
-        <v>151.75</v>
-      </c>
-      <c r="U2" t="n">
-        <v>6.34</v>
-      </c>
-      <c r="V2" t="n">
-        <v>13.84</v>
-      </c>
-      <c r="W2" t="n">
-        <v>29.44</v>
+        <v>66.29000000000001</v>
       </c>
       <c r="AA2" t="n">
-        <v>57.4</v>
+        <v>26.8</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -774,329 +762,269 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/alpine-texworld-limited-prospectus_103604.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/tablespace-technologies-limited-drhp_103710.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Abridged%20prospectus_p.pdf</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>Alpine Texworld Ltd.</t>
-        </is>
-      </c>
-      <c r="AI2" t="n">
-        <v>224</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>29.44</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>68.56</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/alpine-texworld-ltd</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/TABLESPACE%20TECHNOLOGIES%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGS Health Limited</t>
+          <t>Shiprocket Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Healthcare Services</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>2041.42</v>
-      </c>
-      <c r="R3" t="n">
-        <v>70.84999999999999</v>
-      </c>
-      <c r="S3" t="n">
-        <v>206.95</v>
-      </c>
-      <c r="T3" t="n">
-        <v>44.79</v>
-      </c>
-      <c r="U3" t="n">
-        <v>10.14</v>
-      </c>
-      <c r="V3" t="n">
-        <v>4</v>
-      </c>
-      <c r="W3" t="n">
-        <v>4.55</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>54.6</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/ags-health-limited-udrhp_103617.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/AGS%20Health%20Limited%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/shiprocket-limited-prospectus_103843.html</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Shiprocket Ltd.</t>
+        </is>
+      </c>
+      <c r="AI3" t="n">
+        <v>10230</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>99.02</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>88.64</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>45</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/shiprocket-ltd</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zetwerk Manufacturing Businesses Limited</t>
+          <t>Lalithaa Jewellery Mart Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>96837455</v>
-      </c>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>15913.32</v>
-      </c>
-      <c r="R4" t="n">
-        <v>40.43</v>
-      </c>
-      <c r="V4" t="n">
-        <v>-2.22</v>
-      </c>
-      <c r="W4" t="n">
-        <v>21.11</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>47.7</v>
+          <t>Jewellery</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/zetwerk-manufacturing-businesses-limited-udrhp_103643.html</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Zetwerk%20Manufacturing%20Businesses%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/lalithaa-jewellery-mart-limited-prospectus_103788.html</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Lalithaa Jewellery Mart Ltd.</t>
+        </is>
+      </c>
+      <c r="AI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>82.84999999999999</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>62.73</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>145.38</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>73.77</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>11.38</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/lalithaa-jewellery-mart-ltd</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Beauty Garage Limited</t>
+          <t>Lumino Industries Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R5" t="n">
-        <v>-99.79000000000001</v>
-      </c>
-      <c r="V5" t="n">
-        <v>43.33</v>
-      </c>
-      <c r="W5" t="n">
-        <v>55.04</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>15</v>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Diversified Industrials</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>MONITOR</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/beauty-garage-limited-drhp_103479.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/BEAUTY%20GARAGE%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/lumino-industries-limited-corrigendum-to-drhp_103755.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tonbo Imaging India Limited</t>
+          <t>Dhoot Transmission Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Capital Goods</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1117,39 +1045,76 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/tonbo-imaging-india-limited_103625.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/dhoot-transmission-limited_103722.html</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Dhoot Transmission Ltd.</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>30285</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>16.29</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>82.78</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>212.92</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>51.88</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>37.77</v>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/dhoot-transmission-ltd</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sillverton Industries Limited</t>
+          <t>Juniper Green Energy Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1159,7 +1124,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1170,140 +1135,44 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/sillverton-industries-limited-addendum-ii_103621.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>J Pan Tubular Components Limited</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/j-pan-tubular-components-limited_103499.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LEAP India Limited</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/leap-india-limited-prospectus_103511.html</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>Leap India Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>6392</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>6.19</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>55.64</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>16.84</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>12.62</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>4.34</v>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/leap-india-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/juniper-green-energy-limited-prospectus_103747.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Juniper Green Energy Ltd.</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>15110</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>85.94</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/juniper-green-energy-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: weekly DRHP/IPO monitor refresh (2026-08-31)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR7"/>
+  <dimension ref="A1:AR12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tablespace Technologies Limited</t>
+          <t>Avaada Electro Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>UDRHP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>IT Services</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -732,17 +732,38 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="I2" t="n">
+        <v>529.05</v>
+      </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q2" t="n">
-        <v>2262.29</v>
+        <v>5303.52</v>
       </c>
       <c r="R2" t="n">
-        <v>66.29000000000001</v>
+        <v>481.77</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="T2" t="n">
+        <v>-11.63</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="V2" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="W2" t="n">
+        <v>81.51000000000001</v>
+      </c>
+      <c r="X2" t="n">
+        <v>26.68</v>
       </c>
       <c r="AA2" t="n">
-        <v>26.8</v>
+        <v>65</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -751,7 +772,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -762,134 +783,180 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/tablespace-technologies-limited-drhp_103710.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/avaada-electro-limited-udrhp_104034.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/TABLESPACE%20TECHNOLOGIES%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Avaada%20Electro%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shiprocket Limited</t>
+          <t>Jay Jagdamba Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Metals</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>600</v>
+      </c>
+      <c r="J3" t="n">
+        <v>600</v>
+      </c>
+      <c r="L3" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="N3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>3194.36</v>
+      </c>
+      <c r="R3" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="S3" t="n">
+        <v>261.92</v>
+      </c>
+      <c r="T3" t="n">
+        <v>62.69</v>
+      </c>
+      <c r="U3" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="W3" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>60.3</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/shiprocket-limited-prospectus_103843.html</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>Shiprocket Ltd.</t>
-        </is>
-      </c>
-      <c r="AI3" t="n">
-        <v>10230</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>99.02</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>122.8</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>88.64</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>45</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>35.05</v>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/shiprocket-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/jay-jagdamba-limited-udrhp_103937.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Jay%20Jagdamba%20Limited%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lalithaa Jewellery Mart Limited</t>
+          <t>M P Steel (India) Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Jewellery</t>
-        </is>
+          <t>Metals</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>2307290</v>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>413.41</v>
+      </c>
+      <c r="R4" t="n">
+        <v>27.03</v>
+      </c>
+      <c r="S4" t="n">
+        <v>15.81</v>
+      </c>
+      <c r="T4" t="n">
+        <v>139.13</v>
+      </c>
+      <c r="U4" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="V4" t="n">
+        <v>8.17</v>
+      </c>
+      <c r="W4" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>47.4</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -899,64 +966,35 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/lalithaa-jewellery-mart-limited-prospectus_103788.html</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>Lalithaa Jewellery Mart Ltd.</t>
-        </is>
-      </c>
-      <c r="AI4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>34.47</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>82.84999999999999</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>62.73</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>145.38</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>73.77</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>11.38</v>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lalithaa-jewellery-mart-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/m-p-steel-india-limited-drhp_103990.html</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/MPSteel-Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lumino Industries Limited</t>
+          <t>Atomberg Technologies Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -966,55 +1004,86 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Diversified Industrials</t>
-        </is>
+          <t>IT Services</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>76541851</v>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1293.77</v>
+      </c>
+      <c r="R5" t="n">
+        <v>34.84</v>
+      </c>
+      <c r="V5" t="n">
+        <v>-2.55</v>
+      </c>
+      <c r="W5" t="n">
+        <v>67.05</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>38.9</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/lumino-industries-limited-corrigendum-to-drhp_103755.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/atomberg-technologies-limited-drhp_104037.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/ATOMBERG%20TECHNOLOGIES%20LIMITED%20-%20AP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dhoot Transmission Limited</t>
+          <t>Nobel Hygiene Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1024,12 +1093,44 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
-        </is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>846.75</v>
+      </c>
+      <c r="R6" t="n">
+        <v>14.56</v>
+      </c>
+      <c r="S6" t="n">
+        <v>18.91</v>
+      </c>
+      <c r="T6" t="n">
+        <v>8193.42</v>
+      </c>
+      <c r="U6" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="V6" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="W6" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>32.5</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1039,82 +1140,50 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/dhoot-transmission-limited_103722.html</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>Dhoot Transmission Ltd.</t>
-        </is>
-      </c>
-      <c r="AI6" t="n">
-        <v>30285</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>16.29</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>82.78</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>74.09999999999999</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>212.92</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>51.88</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>7.93</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>37.77</v>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/dhoot-transmission-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/nobel-hygiene-limited-drhp_103938.html</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Nobel%20Hygiene%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Juniper Green Energy Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1124,7 +1193,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1135,44 +1204,355 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/juniper-green-energy-limited-prospectus_103747.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Juniper Green Energy Ltd.</t>
-        </is>
-      </c>
-      <c r="AI7" t="n">
-        <v>15110</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>4.02</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>85.94</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>7.93</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>8.890000000000001</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/juniper-green-energy-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hero-motors-limited-addendum-to-drhp_104121.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Annu Projects Limited</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/annu-projects-limited-prospectus_104111.html</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Annu Projects Ltd</t>
+        </is>
+      </c>
+      <c r="AM8" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/annu-projects-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Skyways Air Services Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/skyways-air-services-limited-prospectus_104108.html</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Skyways Air Services Ltd</t>
+        </is>
+      </c>
+      <c r="AM9" t="n">
+        <v>71.11</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>139.69</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>25.13</v>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/skyways-air-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Hy Tech Engineers Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hy-tech-engineers-limited-prospectus_104093.html</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Hy-Tech Engineers Ltd</t>
+        </is>
+      </c>
+      <c r="AM10" t="n">
+        <v>243.84</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>255.77</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>402.08</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>169.54</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/hy-tech-engineers-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Karamtara Engineering Limited</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/karamtara-engineering-limited-addendum-to-drhp_104033.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Augmont Enterprises Limited</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/augmont-enterprises-limited-prospectus_104039.html</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>Augmont Enterprises Ltd.</t>
+        </is>
+      </c>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>36.82</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>81.91</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>105.51</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>226.96</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>121.38</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/augmont-enterprises-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-05)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR12"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,17 +699,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Avaada Electro Limited</t>
+          <t>Kataria Dhulchand Pannalal Jewellers Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -732,38 +732,32 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>529.05</v>
-      </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>5303.52</v>
+        <v>477.87</v>
       </c>
       <c r="R2" t="n">
-        <v>481.77</v>
+        <v>49.12</v>
       </c>
       <c r="S2" t="n">
-        <v>1.64</v>
+        <v>44.55</v>
       </c>
       <c r="T2" t="n">
-        <v>-11.63</v>
+        <v>239.79</v>
       </c>
       <c r="U2" t="n">
-        <v>0.03</v>
+        <v>9.32</v>
       </c>
       <c r="V2" t="n">
-        <v>23.74</v>
+        <v>14.43</v>
       </c>
       <c r="W2" t="n">
-        <v>81.51000000000001</v>
-      </c>
-      <c r="X2" t="n">
-        <v>26.68</v>
+        <v>37.44</v>
       </c>
       <c r="AA2" t="n">
-        <v>65</v>
+        <v>60.8</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -772,7 +766,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -783,29 +777,29 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/avaada-electro-limited-udrhp_104034.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kataria-dhulchand-pannalal-jewellers-limited-drhp_104178.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Avaada%20Electro%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Kataria%20Dhulchand%20Pannalal%20Jewellers%20Ltd%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jay Jagdamba Limited</t>
+          <t>Aragen Life Sciences Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -815,51 +809,48 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
-      </c>
-      <c r="H3" t="n">
-        <v>600</v>
-      </c>
-      <c r="J3" t="n">
-        <v>600</v>
-      </c>
-      <c r="L3" t="n">
-        <v>15000000</v>
       </c>
       <c r="N3" t="n">
         <v>10</v>
       </c>
       <c r="Q3" t="n">
-        <v>3194.36</v>
+        <v>2178.39</v>
       </c>
       <c r="R3" t="n">
-        <v>44.38</v>
+        <v>21683.92</v>
       </c>
       <c r="S3" t="n">
-        <v>261.92</v>
+        <v>1.18</v>
       </c>
       <c r="T3" t="n">
-        <v>62.69</v>
+        <v>20.96</v>
       </c>
       <c r="U3" t="n">
-        <v>8.199999999999999</v>
+        <v>0.05</v>
+      </c>
+      <c r="V3" t="n">
+        <v>27.8</v>
       </c>
       <c r="W3" t="n">
-        <v>12.54</v>
+        <v>11.96</v>
+      </c>
+      <c r="X3" t="n">
+        <v>18.18</v>
       </c>
       <c r="AA3" t="n">
-        <v>60.3</v>
+        <v>52.5</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -868,7 +859,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -879,24 +870,24 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/jay-jagdamba-limited-udrhp_103937.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/aragen-life-sciences-limited-drhp_104157.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Jay%20Jagdamba%20Limited%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/ARAGEN%20LIFE%20SCIENCES%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M P Steel (India) Limited</t>
+          <t>Sembcorp Green Infra Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -911,48 +902,45 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Metals</t>
+          <t>Renewables</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>2307290</v>
-      </c>
-      <c r="N4" t="n">
-        <v>10</v>
+          <t>Fresh</t>
+        </is>
       </c>
       <c r="Q4" t="n">
-        <v>413.41</v>
+        <v>2652.5</v>
       </c>
       <c r="R4" t="n">
-        <v>27.03</v>
+        <v>14.42</v>
       </c>
       <c r="S4" t="n">
-        <v>15.81</v>
+        <v>371.08</v>
       </c>
       <c r="T4" t="n">
-        <v>139.13</v>
+        <v>24.18</v>
       </c>
       <c r="U4" t="n">
-        <v>3.99</v>
+        <v>13.12</v>
       </c>
       <c r="V4" t="n">
-        <v>8.17</v>
+        <v>74.2</v>
       </c>
       <c r="W4" t="n">
-        <v>15.18</v>
+        <v>3.71</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>100</v>
       </c>
       <c r="AA4" t="n">
-        <v>47.4</v>
+        <v>42</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -972,108 +960,77 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/m-p-steel-india-limited-drhp_103990.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sembcorp-green-infra-limited-drhp_104162.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/MPSteel-Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Sembcorp%20Green%20Infra%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atomberg Technologies Limited</t>
+          <t>Gaurik Fashions Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>IT Services</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>76541851</v>
-      </c>
-      <c r="N5" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>1293.77</v>
-      </c>
-      <c r="R5" t="n">
-        <v>34.84</v>
-      </c>
-      <c r="V5" t="n">
-        <v>-2.55</v>
-      </c>
-      <c r="W5" t="n">
-        <v>67.05</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>38.9</v>
+          <t>Apparel</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/atomberg-technologies-limited-drhp_104037.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/ATOMBERG%20TECHNOLOGIES%20LIMITED%20-%20AP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nobel Hygiene Limited</t>
+          <t>India Exposition Mart Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1088,49 +1045,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Manufacturing</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>846.75</v>
-      </c>
-      <c r="R6" t="n">
-        <v>14.56</v>
-      </c>
-      <c r="S6" t="n">
-        <v>18.91</v>
-      </c>
-      <c r="T6" t="n">
-        <v>8193.42</v>
-      </c>
-      <c r="U6" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="V6" t="n">
-        <v>10.01</v>
-      </c>
-      <c r="W6" t="n">
-        <v>5.08</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>32.5</v>
+          <t>Unclassified</t>
+        </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1140,50 +1060,45 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/nobel-hygiene-limited-drhp_103938.html</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/aug-2026/Nobel%20Hygiene%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Priority Jewels Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Automobiles</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1193,7 +1108,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1204,14 +1119,48 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hero-motors-limited-addendum-to-drhp_104121.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/priority-jewels-limited-prospectus_104198.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Priority Jewels Ltd.</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>99.23999999999999</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>39.87</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>166.3</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>104.43</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>15</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/priority-jewels-ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Annu Projects Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1221,17 +1170,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1241,7 +1195,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1252,41 +1206,19 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/annu-projects-limited-prospectus_104111.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Annu Projects Ltd</t>
-        </is>
-      </c>
-      <c r="AM8" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/annu-projects-ipo</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hero-motors-limited-addendum-to-drhp_104121.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Skyways Air Services Limited</t>
+          <t>Annu Projects Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1322,237 +1254,44 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/skyways-air-services-limited-prospectus_104108.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/annu-projects-limited-prospectus_104111.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Skyways Air Services Ltd</t>
-        </is>
+          <t>Annu Projects Ltd.</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>485</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>21.27</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>65.05</v>
       </c>
       <c r="AM9" t="n">
-        <v>71.11</v>
+        <v>2.9</v>
       </c>
       <c r="AN9" t="n">
-        <v>139.69</v>
+        <v>1.72</v>
       </c>
       <c r="AO9" t="n">
-        <v>87.2</v>
+        <v>3.54</v>
       </c>
       <c r="AP9" t="n">
-        <v>25.13</v>
+        <v>2.62</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>-27.27</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/skyways-air-ipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Hy Tech Engineers Limited</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hy-tech-engineers-limited-prospectus_104093.html</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Hy-Tech Engineers Ltd</t>
-        </is>
-      </c>
-      <c r="AM10" t="n">
-        <v>243.84</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>255.77</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>402.08</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>169.54</v>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/hy-tech-engineers-ipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Karamtara Engineering Limited</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Addendum</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/karamtara-engineering-limited-addendum-to-drhp_104033.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Augmont Enterprises Limited</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/augmont-enterprises-limited-prospectus_104039.html</t>
-        </is>
-      </c>
-      <c r="AH12" t="inlineStr">
-        <is>
-          <t>Augmont Enterprises Ltd.</t>
-        </is>
-      </c>
-      <c r="AI12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ12" t="n">
-        <v>36.82</v>
-      </c>
-      <c r="AK12" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>81.91</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>105.51</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>226.96</v>
-      </c>
-      <c r="AO12" t="n">
-        <v>121.38</v>
-      </c>
-      <c r="AP12" t="n">
-        <v>30.49</v>
-      </c>
-      <c r="AQ12" t="n">
-        <v>21.95</v>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/augmont-enterprises-ltd</t>
+          <t>https://groww.in/stocks/annu-projects-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-07)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -882,65 +882,65 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sembcorp Green Infra Limited</t>
+          <t>Lumino Industries Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Renewables</t>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Fresh</t>
-        </is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>5</v>
       </c>
       <c r="Q4" t="n">
-        <v>2652.5</v>
+        <v>202.6</v>
       </c>
       <c r="R4" t="n">
-        <v>14.42</v>
+        <v>0.05</v>
       </c>
       <c r="S4" t="n">
-        <v>371.08</v>
+        <v>160</v>
       </c>
       <c r="T4" t="n">
-        <v>24.18</v>
+        <v>28.42</v>
       </c>
       <c r="U4" t="n">
-        <v>13.12</v>
-      </c>
-      <c r="V4" t="n">
-        <v>74.2</v>
+        <v>7.66</v>
       </c>
       <c r="W4" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>100</v>
+        <v>24.61</v>
+      </c>
+      <c r="X4" t="n">
+        <v>25.75</v>
       </c>
       <c r="AA4" t="n">
-        <v>42</v>
+        <v>48.7</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -960,29 +960,66 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sembcorp-green-infra-limited-drhp_104162.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lumino-industries-limited-prospectus_104288.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Sembcorp%20Green%20Infra%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Lumino%20Industries%20Limited%20-%20Abridged%20Prospectus_p.pdf</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Lumino Industries Ltd.</t>
+        </is>
+      </c>
+      <c r="AI4" t="n">
+        <v>3488</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>71.97</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>50.48</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>33.18</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>130.83</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>34.15</v>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/lumino-industries-ltd</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gaurik Fashions Limited</t>
+          <t>Sembcorp Green Infra Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -992,40 +1029,77 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Apparel</t>
-        </is>
+          <t>Renewables</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>2652.5</v>
+      </c>
+      <c r="R5" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="S5" t="n">
+        <v>371.08</v>
+      </c>
+      <c r="T5" t="n">
+        <v>24.18</v>
+      </c>
+      <c r="U5" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="V5" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="W5" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>42</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sembcorp-green-infra-limited-drhp_104162.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Sembcorp%20Green%20Infra%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>India Exposition Mart Limited</t>
+          <t>Mahanadi Coalfields Ltd.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1048,9 +1122,32 @@
           <t>Unclassified</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OFS</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="M6" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-99.88</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1060,35 +1157,40 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Priority Jewels Limited</t>
+          <t>Gaurik Fashions Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1098,7 +1200,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Apparel</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1108,7 +1210,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1119,58 +1221,24 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/priority-jewels-limited-prospectus_104198.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Priority Jewels Ltd.</t>
-        </is>
-      </c>
-      <c r="AI7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>99.23999999999999</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>39.87</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>166.3</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>104.43</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>15</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/priority-jewels-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>India Exposition Mart Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1180,12 +1248,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1195,7 +1258,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1206,19 +1269,19 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/hero-motors-limited-addendum-to-drhp_104121.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Annu Projects Limited</t>
+          <t>Deepa Jewellers Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1233,7 +1296,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1254,44 +1322,119 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/aug-2026/annu-projects-limited-prospectus_104111.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Annu Projects Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>485</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>21.27</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>65.05</v>
+          <t>Deepa Jewellers Ltd</t>
+        </is>
       </c>
       <c r="AM9" t="n">
-        <v>2.9</v>
+        <v>42.2</v>
       </c>
       <c r="AN9" t="n">
-        <v>1.72</v>
+        <v>37</v>
       </c>
       <c r="AO9" t="n">
-        <v>3.54</v>
+        <v>105.69</v>
       </c>
       <c r="AP9" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>-27.27</v>
+        <v>17.86</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/annu-projects-ltd</t>
+          <t>https://groww.in/ipo/deepa-jewellers-ipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Priority Jewels Limited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Prospectus</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>IPO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/priority-jewels-limited-prospectus_104198.html</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Priority Jewels Ltd.</t>
+        </is>
+      </c>
+      <c r="AI10" t="n">
+        <v>426</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>70</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>99.23999999999999</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>39.87</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>166.3</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>104.43</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>15</v>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/priority-jewels-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-08)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR10"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -699,32 +699,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kataria Dhulchand Pannalal Jewellers Limited</t>
+          <t>Lumino Industries Limited</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Diversified Industrials</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -733,31 +733,31 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q2" t="n">
-        <v>477.87</v>
+        <v>202.6</v>
       </c>
       <c r="R2" t="n">
-        <v>49.12</v>
+        <v>0.05</v>
       </c>
       <c r="S2" t="n">
-        <v>44.55</v>
+        <v>160</v>
       </c>
       <c r="T2" t="n">
-        <v>239.79</v>
+        <v>28.42</v>
       </c>
       <c r="U2" t="n">
-        <v>9.32</v>
-      </c>
-      <c r="V2" t="n">
-        <v>14.43</v>
+        <v>7.66</v>
       </c>
       <c r="W2" t="n">
-        <v>37.44</v>
+        <v>24.61</v>
+      </c>
+      <c r="X2" t="n">
+        <v>25.75</v>
       </c>
       <c r="AA2" t="n">
-        <v>60.8</v>
+        <v>48.7</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -777,179 +777,162 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/kataria-dhulchand-pannalal-jewellers-limited-drhp_104178.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lumino-industries-limited-prospectus_104288.html</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Kataria%20Dhulchand%20Pannalal%20Jewellers%20Ltd%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Lumino%20Industries%20Limited%20-%20Abridged%20Prospectus_p.pdf</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Lumino Industries Ltd.</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>3496</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>71.97</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>50.48</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>33.18</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>130.83</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>34.15</v>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/lumino-industries-ltd</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aragen Life Sciences Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>2178.39</v>
-      </c>
-      <c r="R3" t="n">
-        <v>21683.92</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="T3" t="n">
-        <v>20.96</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="V3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="W3" t="n">
-        <v>11.96</v>
-      </c>
-      <c r="X3" t="n">
-        <v>18.18</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>52.5</v>
+          <t>Automobiles</t>
+        </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/aragen-life-sciences-limited-drhp_104157.html</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/ARAGEN%20LIFE%20SCIENCES%20LIMITED%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lumino Industries Limited</t>
+          <t>Mahanadi Coalfields Ltd.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Diversified Industrials</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Both</t>
-        </is>
+          <t>OFS</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="M4" t="n">
+        <v>661836300</v>
       </c>
       <c r="N4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q4" t="n">
-        <v>202.6</v>
+        <v>3.71</v>
       </c>
       <c r="R4" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="S4" t="n">
-        <v>160</v>
-      </c>
-      <c r="T4" t="n">
-        <v>28.42</v>
-      </c>
-      <c r="U4" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="W4" t="n">
-        <v>24.61</v>
-      </c>
-      <c r="X4" t="n">
-        <v>25.75</v>
+        <v>-99.88</v>
       </c>
       <c r="AA4" t="n">
-        <v>48.7</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, IPO_STAGE, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -960,146 +943,72 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/lumino-industries-limited-prospectus_104288.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Lumino%20Industries%20Limited%20-%20Abridged%20Prospectus_p.pdf</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>Lumino Industries Ltd.</t>
-        </is>
-      </c>
-      <c r="AI4" t="n">
-        <v>3488</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>21.93</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>71.97</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>50.48</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>33.18</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>130.83</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>27.7</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>34.15</v>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/lumino-industries-ltd</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sembcorp Green Infra Limited</t>
+          <t>Gaurik Fashions Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Renewables</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>2652.5</v>
-      </c>
-      <c r="R5" t="n">
-        <v>14.42</v>
-      </c>
-      <c r="S5" t="n">
-        <v>371.08</v>
-      </c>
-      <c r="T5" t="n">
-        <v>24.18</v>
-      </c>
-      <c r="U5" t="n">
-        <v>13.12</v>
-      </c>
-      <c r="V5" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="W5" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>100</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>42</v>
+          <t>Apparel</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>DIG DEEPER</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/sembcorp-green-infra-limited-drhp_104162.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Sembcorp%20Green%20Infra%20Limited%20-%20Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mahanadi Coalfields Ltd.</t>
+          <t>India Exposition Mart Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1122,32 +1031,9 @@
           <t>Unclassified</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>OFS</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="M6" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="R6" t="n">
-        <v>-99.88</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0</v>
-      </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1157,25 +1043,20 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gaurik Fashions Limited</t>
+          <t>Deepa Jewellers Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1185,12 +1066,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1200,7 +1081,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Apparel</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1210,7 +1091,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1221,29 +1102,63 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Deepa Jewellers Ltd.</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>44.02</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>37</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>105.69</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>17.86</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>24.86</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>https://groww.in/stocks/deepa-jewellers-ltd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>India Exposition Mart Limited</t>
+          <t>Vinod Texworld Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1269,19 +1184,29 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vinod-texworld-limited-prospectus_104299.html</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Vinod Texworld Ltd</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>https://groww.in/ipo/vinod-texworld-ipo</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Deepa Jewellers Limited</t>
+          <t>Priority Jewels Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1322,117 +1247,42 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/priority-jewels-limited-prospectus_104198.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Deepa Jewellers Ltd</t>
-        </is>
+          <t>Priority Jewels Ltd.</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>408</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>70</v>
       </c>
       <c r="AM9" t="n">
-        <v>42.2</v>
+        <v>99.23999999999999</v>
       </c>
       <c r="AN9" t="n">
-        <v>37</v>
+        <v>39.87</v>
       </c>
       <c r="AO9" t="n">
-        <v>105.69</v>
+        <v>166.3</v>
       </c>
       <c r="AP9" t="n">
-        <v>17.86</v>
+        <v>104.43</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>15</v>
       </c>
       <c r="AR9" t="inlineStr">
-        <is>
-          <t>https://groww.in/ipo/deepa-jewellers-ipo</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Priority Jewels Limited</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/priority-jewels-limited-prospectus_104198.html</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Priority Jewels Ltd.</t>
-        </is>
-      </c>
-      <c r="AI10" t="n">
-        <v>426</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>70</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>99.23999999999999</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>39.87</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>166.3</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>104.43</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>15</v>
-      </c>
-      <c r="AR10" t="inlineStr">
         <is>
           <t>https://groww.in/stocks/priority-jewels-ltd</t>
         </is>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-09)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>3496</v>
+        <v>3296</v>
       </c>
       <c r="AJ2" t="n">
         <v>21.93</v>
@@ -826,17 +826,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Torrent Gas Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -846,17 +846,43 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Automobiles</t>
-        </is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>335000000</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1396.78</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-76.45999999999999</v>
+      </c>
+      <c r="S3" t="n">
+        <v>55.68</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-80.18000000000001</v>
+      </c>
+      <c r="U3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -866,96 +892,78 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mahanadi Coalfields Ltd.</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>OFS</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="M4" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="R4" t="n">
-        <v>-99.88</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0</v>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gaurik Fashions Limited</t>
+          <t>Mahanadi Coalfields Ltd.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -965,7 +973,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -975,40 +983,63 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Apparel</t>
-        </is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OFS</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="M5" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="N5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-99.88</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>India Exposition Mart Limited</t>
+          <t>Gaurik Fashions Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1018,17 +1049,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Apparel</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1038,7 +1074,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1049,14 +1085,14 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Deepa Jewellers Limited</t>
+          <t>India Exposition Mart Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1066,22 +1102,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1102,53 +1133,19 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Deepa Jewellers Ltd.</t>
-        </is>
-      </c>
-      <c r="AI7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>44.02</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>37</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>105.69</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>17.86</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>24.86</v>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/deepa-jewellers-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Vinod Texworld Limited</t>
+          <t>Deepa Jewellers Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1163,7 +1160,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1184,29 +1186,56 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vinod-texworld-limited-prospectus_104299.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Vinod Texworld Ltd</t>
-        </is>
+          <t>Deepa Jewellers Ltd.</t>
+        </is>
+      </c>
+      <c r="AI8" t="n">
+        <v>1868</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>44.02</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>72.98</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>37</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>105.69</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>17.86</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>24.86</v>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/vinod-texworld-ipo</t>
+          <t>https://groww.in/stocks/deepa-jewellers-ltd</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Priority Jewels Limited</t>
+          <t>Vinod Texworld Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1221,12 +1250,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1247,44 +1271,29 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/priority-jewels-limited-prospectus_104198.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vinod-texworld-limited-prospectus_104299.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Priority Jewels Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>408</v>
-      </c>
-      <c r="AJ9" t="n">
+          <t>Vinod Texworld Ltd</t>
+        </is>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AN9" t="n">
         <v>0</v>
       </c>
-      <c r="AK9" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>70</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>99.23999999999999</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>39.87</v>
-      </c>
       <c r="AO9" t="n">
-        <v>166.3</v>
+        <v>0</v>
       </c>
       <c r="AP9" t="n">
-        <v>104.43</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>15</v>
+        <v>0.05</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/stocks/priority-jewels-ltd</t>
+          <t>https://groww.in/ipo/vinod-texworld-ipo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-10)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>3296</v>
+        <v>3234</v>
       </c>
       <c r="AJ2" t="n">
         <v>21.93</v>
@@ -910,12 +910,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Incred Holdings Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -930,12 +930,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -956,90 +951,67 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mahanadi Coalfields Ltd.</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>OFS</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="M5" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="N5" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="R5" t="n">
-        <v>-99.88</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0</v>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
+        </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gaurik Fashions Limited</t>
+          <t>Mahanadi Coalfields Ltd.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1049,7 +1021,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1059,40 +1031,63 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Apparel</t>
-        </is>
+          <t>Unclassified</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OFS</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="M6" t="n">
+        <v>661836300</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-99.88</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>India Exposition Mart Limited</t>
+          <t>Gaurik Fashions Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1102,17 +1097,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Addendum</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Apparel</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1133,14 +1133,14 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Deepa Jewellers Limited</t>
+          <t>India Exposition Mart Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1150,22 +1150,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1186,56 +1181,19 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Deepa Jewellers Ltd.</t>
-        </is>
-      </c>
-      <c r="AI8" t="n">
-        <v>1868</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>44.02</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>72.98</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>37</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>105.69</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>17.86</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>24.86</v>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/deepa-jewellers-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vinod Texworld Limited</t>
+          <t>Deepa Jewellers Limited</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1250,7 +1208,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1271,29 +1234,44 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/vinod-texworld-limited-prospectus_104299.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Vinod Texworld Ltd</t>
-        </is>
+          <t>Deepa Jewellers Ltd.</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>1936</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>44.02</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>72.98</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.02</v>
+        <v>42.2</v>
       </c>
       <c r="AN9" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="AO9" t="n">
-        <v>0</v>
+        <v>105.69</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.05</v>
+        <v>17.86</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>24.86</v>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>https://groww.in/ipo/vinod-texworld-ipo</t>
+          <t>https://groww.in/stocks/deepa-jewellers-ltd</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-11)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR9"/>
+  <dimension ref="A1:AR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>3234</v>
+        <v>3286</v>
       </c>
       <c r="AJ2" t="n">
         <v>21.93</v>
@@ -826,12 +826,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Torrent Gas Limited</t>
+          <t>Nopaperforms Solutions Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -846,12 +846,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Oil &amp; Gas</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -859,30 +854,36 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>335000000</v>
+      <c r="N3" t="n">
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>1396.78</v>
+        <v>115.65</v>
       </c>
       <c r="R3" t="n">
-        <v>-76.45999999999999</v>
+        <v>25.24</v>
       </c>
       <c r="S3" t="n">
-        <v>55.68</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>-80.18000000000001</v>
+        <v>408.67</v>
       </c>
       <c r="U3" t="n">
-        <v>3.99</v>
+        <v>0.83</v>
+      </c>
+      <c r="V3" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="W3" t="n">
+        <v>33.12</v>
       </c>
       <c r="AA3" t="n">
-        <v>8.199999999999999</v>
+        <v>48</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -898,29 +899,29 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/nopaperforms-solutions-limited-udrhp-1_104427.html</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/NOPAPERFORMS%20SOLUTIONS%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Incred Holdings Limited</t>
+          <t>Torrent Gas Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -930,12 +931,43 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>335000000</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1396.78</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-76.45999999999999</v>
+      </c>
+      <c r="S4" t="n">
+        <v>55.68</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-80.18000000000001</v>
+      </c>
+      <c r="U4" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -945,30 +977,35 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -978,12 +1015,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1004,29 +1036,29 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mahanadi Coalfields Ltd.</t>
+          <t>Glass Wall Systems (India) Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1034,32 +1066,9 @@
           <t>Unclassified</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>OFS</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="M6" t="n">
-        <v>661836300</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="R6" t="n">
-        <v>-99.88</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0</v>
-      </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>INSUFFICIENT</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1069,35 +1078,30 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>DRHP_PDF, derived</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/mahanadi-coalfields-ltd-drhp_104290.html</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Mahanadi%20Coalfields%20Limited%20_Draft%20Abridged%20Prospectus_p.pdf</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gaurik Fashions Limited</t>
+          <t>Incred Holdings Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>Corrigendum</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1107,12 +1111,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Apparel</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1133,34 +1132,39 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/gaurik-fashions-limited-addendum-to-drhp_104276.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>India Exposition Mart Limited</t>
+          <t>Hero Motors Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>DRHP</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>DRHP</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Unclassified</t>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1170,7 +1174,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -1181,97 +1185,7 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/india-exposition-mart-limited_104273.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Deepa Jewellers Limited</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Prospectus</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>IPO</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Consumer</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>INSUFFICIENT</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>FILED_THIS_WEEK</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/deepa-jewellers-limited-prospectus_104286.html</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>Deepa Jewellers Ltd.</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>1936</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>44.02</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>72.98</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>37</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>105.69</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>17.86</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>24.86</v>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>https://groww.in/stocks/deepa-jewellers-ltd</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: daily DRHP/IPO monitor refresh (2026-09-12)
</commit_message>
<xml_diff>
--- a/data/tracker_appendix.xlsx
+++ b/data/tracker_appendix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR8"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -911,17 +911,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Torrent Gas Limited</t>
+          <t>M K C Agro Fresh Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UDRHP</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -944,35 +944,47 @@
           <t>Both</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>335000000</v>
+      <c r="N4" t="n">
+        <v>10</v>
       </c>
       <c r="Q4" t="n">
-        <v>1396.78</v>
+        <v>521.53</v>
       </c>
       <c r="R4" t="n">
-        <v>-76.45999999999999</v>
+        <v>6.38</v>
       </c>
       <c r="S4" t="n">
-        <v>55.68</v>
+        <v>22.11</v>
       </c>
       <c r="T4" t="n">
-        <v>-80.18000000000001</v>
+        <v>14.09</v>
       </c>
       <c r="U4" t="n">
-        <v>3.99</v>
+        <v>4.24</v>
+      </c>
+      <c r="V4" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="W4" t="n">
+        <v>15.92</v>
+      </c>
+      <c r="X4" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1.47</v>
       </c>
       <c r="AA4" t="n">
-        <v>8.199999999999999</v>
+        <v>30.8</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>DIG DEEPER</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -983,29 +995,29 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/m-k-c-agro-fresh-limited-drhp_104430.html</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/M%20K%20C%20AGRO%20FRESH%20LIMITED%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Runwal Enterprises Limited</t>
+          <t>Torrent Gas Limited</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Addendum</t>
+          <t>UDRHP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1015,12 +1027,43 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Unclassified</t>
-        </is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>335000000</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1396.78</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-76.45999999999999</v>
+      </c>
+      <c r="S5" t="n">
+        <v>55.68</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-80.18000000000001</v>
+      </c>
+      <c r="U5" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>INSUFFICIENT</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1030,20 +1073,25 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DRHP_PDF, derived</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/torrent-gas-limited-udrhp-i_104350.html</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/sebi_data/commondocs/sep-2026/Torrent%20Gas%20Limited%20-%20DAP_p.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Glass Wall Systems (India) Limited</t>
+          <t>Runwal Enterprises Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1053,12 +1101,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prospectus</t>
+          <t>Addendum</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>IPO</t>
+          <t>DRHP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1073,7 +1121,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK</t>
+          <t>FILED_THIS_WEEK, UPDATED</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -1084,29 +1132,29 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/runwal-enterprises-limited-addendum-to-drhp_104424.html</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Incred Holdings Limited</t>
+          <t>Glass Wall Systems (India) Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Corrigendum</t>
+          <t>Prospectus</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DRHP</t>
+          <t>IPO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1121,7 +1169,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>FILED_THIS_WEEK, UPDATED</t>
+          <t>FILED_THIS_WEEK</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -1132,19 +1180,19 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/glass-wall-systems-india-limited-prospectus_104426.html</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hero Motors Limited</t>
+          <t>Incred Holdings Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1159,12 +1207,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Automobiles</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1184,6 +1227,59 @@
       </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/incred-holdings-limited-corrigendum-to-udrhp_104399.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Hero Motors Limited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Corrigendum</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DRHP</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Automobiles</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>FILED_THIS_WEEK, UPDATED</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
         <is>
           <t>https://www.sebi.gov.in/filings/public-issues/sep-2026/hero-motors-limited-corrigendum-to-addendum-_104330.html</t>
         </is>

</xml_diff>